<commit_message>
paradigmFSMs fixed, 1 folder rename
</commit_message>
<xml_diff>
--- a/Paradigms/P0600_mlGym.xlsx
+++ b/Paradigms/P0600_mlGym.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/loaloa/homedataAir/phd/ratvr/VirtualReality/UnityRatVR/Paradigms/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1724609-AA70-1C4C-A059-92C42DDDE7BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFBBA057-D454-AF47-84D1-8FA308F9F551}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4357,7 +4357,7 @@
         <v>80</v>
       </c>
       <c r="L2" s="22" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="M2" s="23"/>
       <c r="N2" s="20" t="s">
@@ -4388,7 +4388,7 @@
         <v>80</v>
       </c>
       <c r="L3" s="22" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="M3" s="23"/>
       <c r="N3" s="20" t="s">
@@ -4417,7 +4417,7 @@
         <v>80</v>
       </c>
       <c r="L4" s="22" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="M4" s="23"/>
       <c r="N4" s="20" t="s">
@@ -4446,7 +4446,7 @@
         <v>80</v>
       </c>
       <c r="L5" s="36" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
       <c r="M5" s="23"/>
       <c r="N5" s="20" t="s">
@@ -4527,9 +4527,8 @@
       <c r="H9" s="48"/>
       <c r="I9" s="48"/>
       <c r="J9" s="3"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="22" t="s">
-        <v>462</v>
+      <c r="K9" s="22" t="s">
+        <v>459</v>
       </c>
       <c r="Q9" s="4"/>
     </row>
@@ -4544,9 +4543,8 @@
       <c r="H10" s="48"/>
       <c r="I10" s="48"/>
       <c r="J10" s="3"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="22" t="s">
-        <v>463</v>
+      <c r="K10" s="22" t="s">
+        <v>460</v>
       </c>
       <c r="Q10" s="4"/>
     </row>
@@ -4560,9 +4558,8 @@
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="3"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="22" t="s">
-        <v>464</v>
+      <c r="K11" s="22" t="s">
+        <v>461</v>
       </c>
       <c r="Q11" s="4"/>
     </row>
@@ -4576,9 +4573,8 @@
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="3"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="36" t="s">
-        <v>465</v>
+      <c r="K12" s="36" t="s">
+        <v>458</v>
       </c>
       <c r="Q12" s="4"/>
     </row>

</xml_diff>

<commit_message>
movement vars clean up
</commit_message>
<xml_diff>
--- a/Paradigms/P0600_mlGym.xlsx
+++ b/Paradigms/P0600_mlGym.xlsx
@@ -8,17 +8,28 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/loaloa/homedataAir/phd/ratvr/VirtualReality/UnityRatVR/Paradigms/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFBBA057-D454-AF47-84D1-8FA308F9F551}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF45F75D-A92B-5647-81D8-E75C166CC2A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Environment" sheetId="1" r:id="rId1"/>
     <sheet name="EnvParameters" sheetId="2" r:id="rId2"/>
     <sheet name="SessionParameters" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
     </ext>
@@ -27,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="468">
   <si>
     <t>x0</t>
   </si>
@@ -1425,6 +1436,12 @@
   </si>
   <si>
     <t>mlTexture_LeftCircle_small</t>
+  </si>
+  <si>
+    <t>none,none2</t>
+  </si>
+  <si>
+    <t>5,0</t>
   </si>
 </sst>
 </file>
@@ -4357,7 +4374,7 @@
         <v>80</v>
       </c>
       <c r="L2" s="22" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="M2" s="23"/>
       <c r="N2" s="20" t="s">
@@ -4388,7 +4405,7 @@
         <v>80</v>
       </c>
       <c r="L3" s="22" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="M3" s="23"/>
       <c r="N3" s="20" t="s">
@@ -4417,14 +4434,14 @@
         <v>80</v>
       </c>
       <c r="L4" s="22" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="M4" s="23"/>
       <c r="N4" s="20" t="s">
         <v>419</v>
       </c>
       <c r="O4" s="21">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P4" s="30"/>
       <c r="R4" s="3"/>
@@ -4446,14 +4463,14 @@
         <v>80</v>
       </c>
       <c r="L5" s="36" t="s">
-        <v>465</v>
+        <v>458</v>
       </c>
       <c r="M5" s="23"/>
       <c r="N5" s="20" t="s">
         <v>421</v>
       </c>
       <c r="O5" s="37">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P5" s="38"/>
       <c r="R5" s="3"/>
@@ -4470,7 +4487,7 @@
       <c r="I6" s="39"/>
       <c r="J6" s="40"/>
       <c r="K6" s="39"/>
-      <c r="L6" s="9"/>
+      <c r="L6" s="5"/>
       <c r="M6" s="41"/>
       <c r="N6" s="40"/>
       <c r="O6" s="39"/>
@@ -4489,7 +4506,6 @@
       <c r="I7" s="39"/>
       <c r="J7" s="40"/>
       <c r="K7" s="39"/>
-      <c r="L7" s="9"/>
       <c r="M7" s="41"/>
       <c r="N7" s="40"/>
       <c r="O7" s="39"/>
@@ -4509,7 +4525,6 @@
       <c r="I8" s="9"/>
       <c r="J8" s="40"/>
       <c r="K8" s="39"/>
-      <c r="L8" s="9"/>
       <c r="M8" s="12"/>
       <c r="N8" s="40"/>
       <c r="O8" s="39"/>
@@ -4527,9 +4542,6 @@
       <c r="H9" s="48"/>
       <c r="I9" s="48"/>
       <c r="J9" s="3"/>
-      <c r="K9" s="22" t="s">
-        <v>459</v>
-      </c>
       <c r="Q9" s="4"/>
     </row>
     <row r="10" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -4543,9 +4555,6 @@
       <c r="H10" s="48"/>
       <c r="I10" s="48"/>
       <c r="J10" s="3"/>
-      <c r="K10" s="22" t="s">
-        <v>460</v>
-      </c>
       <c r="Q10" s="4"/>
     </row>
     <row r="11" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -4559,7 +4568,10 @@
       <c r="I11" s="4"/>
       <c r="J11" s="3"/>
       <c r="K11" s="22" t="s">
-        <v>461</v>
+        <v>459</v>
+      </c>
+      <c r="L11" s="22" t="s">
+        <v>462</v>
       </c>
       <c r="Q11" s="4"/>
     </row>
@@ -4573,8 +4585,11 @@
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="3"/>
-      <c r="K12" s="36" t="s">
-        <v>458</v>
+      <c r="K12" s="22" t="s">
+        <v>460</v>
+      </c>
+      <c r="L12" s="22" t="s">
+        <v>463</v>
       </c>
       <c r="Q12" s="4"/>
     </row>
@@ -4588,8 +4603,12 @@
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
       <c r="J13" s="3"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="4"/>
+      <c r="K13" s="22" t="s">
+        <v>461</v>
+      </c>
+      <c r="L13" s="22" t="s">
+        <v>464</v>
+      </c>
       <c r="Q13" s="4"/>
     </row>
     <row r="14" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -4602,8 +4621,12 @@
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
       <c r="J14" s="3"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="4"/>
+      <c r="K14" s="36" t="s">
+        <v>458</v>
+      </c>
+      <c r="L14" s="36" t="s">
+        <v>465</v>
+      </c>
       <c r="Q14" s="4"/>
     </row>
     <row r="15" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -4616,7 +4639,7 @@
       <c r="H15" s="6"/>
       <c r="J15" s="3"/>
       <c r="K15" s="5"/>
-      <c r="L15" s="4"/>
+      <c r="L15" s="9"/>
       <c r="Q15" s="4"/>
     </row>
     <row r="16" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -4629,7 +4652,7 @@
       <c r="H16" s="6"/>
       <c r="J16" s="3"/>
       <c r="K16" s="5"/>
-      <c r="L16" s="4"/>
+      <c r="L16" s="9"/>
       <c r="Q16" s="4"/>
     </row>
     <row r="17" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -4642,7 +4665,7 @@
       <c r="H17" s="6"/>
       <c r="J17" s="3"/>
       <c r="K17" s="5"/>
-      <c r="L17" s="4"/>
+      <c r="L17" s="9"/>
       <c r="Q17" s="4"/>
     </row>
     <row r="18" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -15688,7 +15711,7 @@
         <v>451</v>
       </c>
       <c r="B12" s="63" t="s">
-        <v>438</v>
+        <v>466</v>
       </c>
       <c r="C12" s="66" t="s">
         <v>452</v>
@@ -15702,8 +15725,8 @@
       <c r="A13" s="65" t="s">
         <v>453</v>
       </c>
-      <c r="B13" s="67">
-        <v>-1</v>
+      <c r="B13" s="67" t="s">
+        <v>467</v>
       </c>
       <c r="C13" s="61"/>
       <c r="D13" s="40"/>

</xml_diff>